<commit_message>
Adjunto diagrama Burndownchart actualizado.
</commit_message>
<xml_diff>
--- a/BurnDownChart - Maply Services.xlsx
+++ b/BurnDownChart - Maply Services.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>Maply Services</t>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>Burn Down Chart</t>
@@ -214,11 +214,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1524599581"/>
-        <c:axId val="1632653548"/>
+        <c:axId val="935879820"/>
+        <c:axId val="2140703375"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1524599581"/>
+        <c:axId val="935879820"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -274,10 +274,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1632653548"/>
+        <c:crossAx val="2140703375"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1632653548"/>
+        <c:axId val="2140703375"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -354,7 +354,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1524599581"/>
+        <c:crossAx val="935879820"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -732,8 +732,8 @@
         <v>46199.0</v>
       </c>
       <c r="B16" s="3"/>
-      <c r="C16" s="3">
-        <v>0.0</v>
+      <c r="C16" s="5">
+        <v>31.0</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -741,7 +741,7 @@
         <v>46206.0</v>
       </c>
       <c r="C17" s="7">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">

</xml_diff>